<commit_message>
Fix Playwright scraper, add safeGoto, update meta/fantasy endpoints
</commit_message>
<xml_diff>
--- a/assets/afl_fixtures_2025_round_24.xlsx
+++ b/assets/afl_fixtures_2025_round_24.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FlutterProjects\my_app\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA3AB75-EE3C-4C65-87EE-E07286CD40A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F5E6AC-1970-417E-B25A-CC8FA84C72F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{9374563A-F70D-41F6-AA26-ACBFD3D87333}"/>
   </bookViews>
   <sheets>
-    <sheet name="AFL 2026 Fixtures" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AFL 2026 Fixtures'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$B$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
   <si>
     <t xml:space="preserve">Sydney Swans </t>
   </si>
@@ -201,6 +201,39 @@
   </si>
   <si>
     <t>https://www.afl.com.au/afl/matches/7163</t>
+  </si>
+  <si>
+    <t>Match ID</t>
+  </si>
+  <si>
+    <t>CD_M20250142407</t>
+  </si>
+  <si>
+    <t>CD_M20250142405</t>
+  </si>
+  <si>
+    <t>CD_M20250142401</t>
+  </si>
+  <si>
+    <t>CD_M20250142403</t>
+  </si>
+  <si>
+    <t>CD_M20250142406</t>
+  </si>
+  <si>
+    <t>CD_M20250142408</t>
+  </si>
+  <si>
+    <t>CD_M20250142402</t>
+  </si>
+  <si>
+    <t>CD_M20250142404</t>
+  </si>
+  <si>
+    <t>CD_M20250142409</t>
+  </si>
+  <si>
+    <t>SEASON</t>
   </si>
 </sst>
 </file>
@@ -641,252 +674,312 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D57401C0-0D7F-465C-819C-F6F6EABA98A5}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>28</v>
       </c>
+      <c r="I1" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>37</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>42</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>43</v>
       </c>
+      <c r="I2" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>37</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>44</v>
       </c>
+      <c r="I3" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>34</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>40</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>25</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>45</v>
       </c>
+      <c r="I4" t="s">
+        <v>57</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2025</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>35</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>36</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>46</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>47</v>
       </c>
+      <c r="I5" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>37</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>24</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>48</v>
       </c>
+      <c r="I6" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2025</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>0</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>38</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>22</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>49</v>
       </c>
+      <c r="I7" t="s">
+        <v>60</v>
+      </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2025</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>7</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>39</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>51</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>50</v>
       </c>
+      <c r="I8" t="s">
+        <v>61</v>
+      </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>6</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>9</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>36</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>52</v>
       </c>
+      <c r="I9" t="s">
+        <v>62</v>
+      </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2025</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>10</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>2</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>41</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>23</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>53</v>
+      </c>
+      <c r="I10" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G10" xr:uid="{D57401C0-0D7F-465C-819C-F6F6EABA98A5}"/>
+  <autoFilter ref="B1:H10" xr:uid="{D57401C0-0D7F-465C-819C-F6F6EABA98A5}"/>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G1048576">
+  <conditionalFormatting sqref="H2:H1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="6"/>
     <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>

</xml_diff>